<commit_message>
bom(xiao): Amazon/AliExpress buy links, add display lens line
Link 1 = Amazon, Link 2 = AliExpress (Scott's preference); the XIAO keeps
Seeed first with Amazon second, and the board keeps JLCPCB/PCBWay. Digi-Key
links dropped: nobody building this orders there. The Mfr part no. column
keeps the reference part each footprint was drawn for, rather than being
replaced by marketplace titles, so a listing can still be checked against it.

Fit caveats flagged in Notes rather than swapped silently: the uxcell switch
lists 6.5 mm pin pitch vs the footprint's 7.0 mm; socket body height and the
Amazon C1 kit's dimensions are unverified. New LENS1-5 line (Scott's watch
crystal listing): diameter not chosen, set by the enclosure bezel. Rows with
an unresolved value are highlighted in the xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
+++ b/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
@@ -10,7 +10,7 @@
     <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$J$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$J$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -551,12 +551,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>https://thepihut.com/products/seeed-xiao-esp32s3-plus</t>
+          <t>https://www.amazon.com/dp/B0H6XJGN3Z</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Plus boards ship WITHOUT pin headers: see the header and socket lines below. Mounted on the back, on sockets.</t>
+          <t>Plus boards ship WITHOUT pin headers: see the header and socket lines below. Mounted on the back, on sockets. The plain XIAO ESP32-S3 (https://www.amazon.com/dp/B0BYSB66S5) is interchangeable and runs the same 8 MB binary. AliExpress: https://www.aliexpress.us/item/3256808599305867.html</t>
         </is>
       </c>
     </row>
@@ -594,61 +594,61 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/MTDELE-Display-Compatible-Arduino-Interfac/dp/B0DJ13VW73</t>
+          <t>https://www.amazon.com/dp/B0DJ13VW73</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/AITRIP-1-28-Display-Multicolored-Arduino/dp/B0H6RQ4C54</t>
+          <t>https://www.aliexpress.us/item/3256813175276825.html</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Check the listing's pin order before buying; the footprint is pad 1 = VCC (+5V) .. pad 7 = RST. The module's own male header plugs into the female socket below.</t>
+          <t>Check the listing's pin order before buying; the footprint is pad 1 = VCC (+5V) .. pad 7 = RST. The module's own male header plugs into the female socket below. Lit area ~32.5 mm dia (docs/DISPLAY-EDGE-TEST.md).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>J (displays)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>LENS1-LENS5</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Female socket 1x07, 2.54 mm, straight</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>8.5 mm body, through hole</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>PinSocket_1x07_P2.54mm_Vertical (in GC9A01_SOCKET)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Sullins PPTC071LFBN-RC</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/sullins-connector-solutions/PPTC071LFBN-RC/810146</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Not a schematic part: modeled inside the display footprint. 8.5 mm is the lift the 3D assumes.</t>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Display lens: mineral watch crystal, double dome</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>2.0 mm thick; DIAMETER NOT CHOSEN (26-45 mm offered)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>enclosure part, no footprint</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>generic</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256806569387664.html</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Diameter is set by the enclosure bezel, not chosen yet; must clear the ~32.5 mm lit area. Pick the size option on the listing. No Amazon source found yet.</t>
         </is>
       </c>
     </row>
@@ -658,11 +658,11 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>J (XIAO)</t>
+          <t>J (displays)</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -676,23 +676,27 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>in XIAO-ESP32-S3-SOCKET</t>
+          <t>PinSocket_1x07_P2.54mm_Vertical (in GC9A01_SOCKET)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sullins PPTC071LFBN-RC</t>
+          <t>Sullins PPTC071LFBN-RC (reference)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/sullins-connector-solutions/PPTC071LFBN-RC/810146</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+          <t>https://www.amazon.com/dp/B0GM7T6XWP</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256812879331298.html</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Same part as the display sockets; 7 per board in all.</t>
+          <t>Not a schematic part: modeled inside the display footprint. 8.5 mm is the lift the 3D assumes; the marketplace sockets' body height is NOT verified. On AliExpress choose the 7P option.</t>
         </is>
       </c>
     </row>
@@ -702,7 +706,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>P (XIAO)</t>
+          <t>J (XIAO)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -710,12 +714,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Male header 1x07, 2.54 mm</t>
+          <t>Female socket 1x07, 2.54 mm, straight</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>cut from a 1x40 breakaway strip (1 strip = 5 sets)</t>
+          <t>8.5 mm body, through hole</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -725,18 +729,22 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Sullins PRPC040SAAN-RC</t>
+          <t>Sullins PPTC071LFBN-RC (reference)</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/sullins-connector-solutions/PRPC040SAAN-RC/2775214</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+          <t>https://www.amazon.com/dp/B0GM7T6XWP</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256812879331298.html</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Soldered to the XIAO, plugs into the XIAO sockets.</t>
+          <t>Same part as the display sockets; 7 per board in all.</t>
         </is>
       </c>
     </row>
@@ -746,45 +754,45 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SW1-SW3</t>
+          <t>P (XIAO)</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Tactile switch, right angle, 6x6 mm</t>
+          <t>Male header 1x07, 2.54 mm</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>SPST-NO, through hole, side actuated</t>
+          <t>cut from a 1x40 breakaway strip (1 strip = 5 sets)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>SW_Tactile_SPST_Angled_PTS645Vx39-2LFS</t>
+          <t>in XIAO-ESP32-S3-SOCKET</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>C&amp;K PTS645VL39-2 LFS</t>
+          <t>Sullins PRPC040SAAN-RC (reference)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/c-k/PTS645VL39-2-LFS/1146765</t>
+          <t>https://www.amazon.com/dp/B0FRZW75VS</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>https://lcsc.com/product-detail/Tactile-Switches_C-K-PTS645VL392LFS_C285523.html</t>
+          <t>https://www.aliexpress.us/item/3256806779943089.html</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Footprint is the C&amp;K part. The uxcell 6x6x8 right-angle switches in the README are NOT verified to fit this footprint.</t>
+          <t>Soldered to the XIAO, plugs into the XIAO sockets.</t>
         </is>
       </c>
     </row>
@@ -794,93 +802,93 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
+          <t>SW1-SW3</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Tactile switch, right angle, 6x6 mm</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>SPST-NO, through hole, side actuated</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>SW_Tactile_SPST_Angled_PTS645Vx39-2LFS</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>C&amp;K PTS645VL39-2 LFS (footprint part)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B008DS13P2</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256810140983087.html</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>FIT NOT VERIFIED: the footprint is the C&amp;K part (7.0 mm mounting-pin pitch); the uxcell 6x6x8 on Amazon lists 6.5 mm. Check one against the board before buying a lot. Exact part: https://lcsc.com/product-detail/Tactile-Switches_C-K-PTS645VL392LFS_C285523.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Electrolytic capacitor, +5V bulk</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>VALUE NOT IN SCHEMATIC - suggested 100 uF 16 V, 6.3 mm dia, 2.5 mm pitch</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>CP_Radial_D6.3mm_P2.50mm</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Panasonic EEU-FC1C101H (suggested)</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/EEU-FC1C101H/2689573</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/EEU-FC1C101/356102</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>Schematic Value field holds the symbol name only - pick and record a value. EEU-FC1C101H is 12.2 mm tall on the back side; check enclosure clearance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Ceramic capacitor 1 uF</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>50 V X7R, radial, 5.08 mm lead spacing</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>C_Disc_D5.0mm_W2.5mm_P5.00mm</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>KEMET C330C105K5R5TA7301</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/kemet/C330C105K5R5TA7301/399-9886-1-ND/3726180</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.digikey.com/en/products/detail/kyocera-avx/SE015C105KAR/2060741</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Display RST hold-off with R1.</t>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0CPDF3HHB</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256812824344961.html</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Schematic Value field holds the symbol name only - pick and record a value. The Amazon kit lists no dimensions: check 6.3 mm dia / 2.5 mm pitch. AliExpress is Nichicon 6.3x7. Height is on the back side; check enclosure clearance.</t>
         </is>
       </c>
     </row>
@@ -890,7 +898,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -898,37 +906,37 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Resistor 10k</t>
+          <t>Ceramic capacitor 1 uF (105)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>1/4 W 5 % carbon film, axial, 10.16 mm pitch</t>
+          <t>50 V, radial, 5.08 mm lead spacing</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
+          <t>C_Disc_D5.0mm_W2.5mm_P5.00mm</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Stackpole CF14JT10K0</t>
+          <t>KEMET C330C105K5R5TA7301 (reference)</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/CF14JT10K0/1741265</t>
+          <t>https://www.amazon.com/dp/B08BF91KY3</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/CFM14JT10K0/1742061</t>
+          <t>https://www.aliexpress.us/item/3256811560978404.html</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Display RST pull-up to 3V3.</t>
+          <t>Display RST hold-off with R1. Both listings are 5.08 mm pitch.</t>
         </is>
       </c>
     </row>
@@ -938,41 +946,45 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>H1-H7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>M3 screw (mounting)</t>
+          <t>Resistor 10k</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>M3-0.5, socket head; 3.2 mm holes</t>
+          <t>1/4 W 5 % carbon film, axial, 10.16 mm pitch</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Edge.Cuts circles, no footprint</t>
+          <t>R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>M3 x 6 DIN 912 (length depends on the enclosure)</t>
+          <t>Stackpole CF14JT10K0 (reference)</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>https://www.aspenfasteners.com/m3-0-5-x-6mm-din-912-iso-4762-metric-socket-head-cap-screws-hex-socket-drive-class-12-9-steel-plain-unbrako/</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+          <t>https://www.amazon.com/dp/B0CL9KXXZB</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256807898146236.html</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Standoffs/length set by the enclosure, not chosen yet.</t>
+          <t>Display RST pull-up to 3V3.</t>
         </is>
       </c>
     </row>
@@ -982,50 +994,98 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>H1-H7</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>M3 screw (mounting)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>M3-0.5, socket head; 3.2 mm holes</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Edge.Cuts circles, no footprint</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>M3 x 6 DIN 912 class 12.9 (length depends on the enclosure)</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DJQH3WSX</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256805704775238.html</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Standoffs/length set by the enclosure, not chosen yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Bare board</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>2 layer, 1.6 mm, 198.82 x 47.78 mm, WHITE solder mask, BLACK silkscreen</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>hot_info_orbs_xiao.kicad_pcb</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>https://jlcpcb.com/quote/pcbOrderFaq/PCB%20Color</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>https://www.pcbway.com/</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Order the colors explicitly: the stackup colors only drive the 3D/STEP, not the gerbers.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:J13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -1033,18 +1093,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
bom(xiao): display lens is 35.5 mm (Scott's pick)
Set by Scott rather than derived from the 32.5 mm lit area: the bezel lip
the crystal seats on is an enclosure dimension, not the BOM's call.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
+++ b/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
@@ -609,46 +609,46 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>LENS1-LENS5</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Display lens: mineral watch crystal, double dome</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>2.0 mm thick; DIAMETER NOT CHOSEN (26-45 mm offered)</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>35.5 mm dia, 2.0 mm thick</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>enclosure part, no footprint</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>generic</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256806569387664.html</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Diameter is set by the enclosure bezel, not chosen yet; must clear the ~32.5 mm lit area. Pick the size option on the listing. No Amazon source found yet.</t>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Choose the Diameter 35.5mm option on the listing (Scott, 2026-10-17); clears the ~32.5 mm lit area. No Amazon source found yet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bom(xiao): plain XIAO ESP32-S3 is the primary part, Plus the alternate
Scott's call: the plain S3 (8 MB flash / 8 MB PSRAM, SKU 113991114) is
enough for the 8 MB binary both boards run, and Seeed sells it with headers
pre-soldered, which removes a soldering step for builders. The Plus stays in
Notes, with its Seeed, Amazon and AliExpress links, for anyone who wants the
16 MB flash. Kept it in one row rather than adding a second U2 row, because
a builder fits one board or the other, never both.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
+++ b/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
@@ -526,12 +526,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Seeed Studio XIAO ESP32-S3 Plus</t>
+          <t>Seeed Studio XIAO ESP32-S3</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ESP32-S3R8, 16 MB flash, 8 MB PSRAM; SKU 102010671</t>
+          <t>ESP32-S3R8, 8 MB flash, 8 MB PSRAM; SKU 113991114</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -541,22 +541,22 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>102010671</t>
+          <t>113991114</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>https://www.seeedstudio.com/Seeed-Studio-XIAO-ESP32S3-Plus-p-6361.html</t>
+          <t>https://www.seeedstudio.com/XIAO-ESP32S3-p-5627.html</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/dp/B0H6XJGN3Z</t>
+          <t>https://www.amazon.com/dp/B0BYSB66S5</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Plus boards ship WITHOUT pin headers: see the header and socket lines below. Mounted on the back, on sockets. The plain XIAO ESP32-S3 (https://www.amazon.com/dp/B0BYSB66S5) is interchangeable and runs the same 8 MB binary. AliExpress: https://www.aliexpress.us/item/3256808599305867.html</t>
+          <t>Primary. Seeed sells it with pin headers Un-Soldered or Pre-Soldered; Pre-Soldered makes the male header line below unnecessary. ALTERNATE if more memory is wanted: XIAO ESP32-S3 Plus (16 MB flash, SKU 102010671) https://www.seeedstudio.com/Seeed-Studio-XIAO-ESP32S3-Plus-p-6361.html / https://www.amazon.com/dp/B0H6XJGN3Z / https://www.aliexpress.us/item/3256808599305867.html - ships WITHOUT headers. Same footprint and the same 8 MB firmware binary on both. Mounted on the back, on sockets.</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Soldered to the XIAO, plugs into the XIAO sockets.</t>
+          <t>Soldered to the XIAO, plugs into the XIAO sockets. Skip if the XIAO was bought Pre-Soldered.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bom(xiao): Link 1 prices and build-cost total; C1 = 100uF 16V
Prices are the Link 1 listings seen live 2026-10-17, so no +40% estimate
mark. Two totals at the bottom: one build bought in whole packs ($104.50:
5 displays from a 3-pack means two packs), and the per-board share with each
pack pro-rated ($55.58). Kept both because the pack-bought figure alone hugely
overstates a club batch, and the pro-rated one alone hides what the first
board really costs. The XIAO-socket line is 0 in build cost because it comes
out of the display sockets' 60-pack. The PCB is left out of both: a JLCPCB
quote depends on quantity and colors, and guessing it would put an estimate
inside a total that is otherwise measured.

C1 value set by Scott and written into the schematic and PCB Value fields;
kicad-cli BOM shows "100uF 16V", DRC 0/0/0 with schematic parity.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
+++ b/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
@@ -10,7 +10,7 @@
     <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$M$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -65,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -74,12 +76,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -457,7 +467,10 @@
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,6 +521,21 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Price (Link 1)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Pack qty</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Build cost</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -554,7 +582,17 @@
           <t>https://www.amazon.com/dp/B0BYSB66S5</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="4" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="4">
+        <f>ROUNDUP(C2/K2,0)*J2</f>
+        <v/>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Primary. Seeed sells it with pin headers Un-Soldered or Pre-Soldered; Pre-Soldered makes the male header line below unnecessary. ALTERNATE if more memory is wanted: XIAO ESP32-S3 Plus (16 MB flash, SKU 102010671) https://www.seeedstudio.com/Seeed-Studio-XIAO-ESP32S3-Plus-p-6361.html / https://www.amazon.com/dp/B0H6XJGN3Z / https://www.aliexpress.us/item/3256808599305867.html - ships WITHOUT headers. Same footprint and the same 8 MB firmware binary on both. Mounted on the back, on sockets.</t>
         </is>
@@ -602,7 +640,17 @@
           <t>https://www.aliexpress.us/item/3256813175276825.html</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" s="4">
+        <f>ROUNDUP(C3/K3,0)*J3</f>
+        <v/>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Check the listing's pin order before buying; the footprint is pad 1 = VCC (+5V) .. pad 7 = RST. The module's own male header plugs into the female socket below. Lit area ~32.5 mm dia (docs/DISPLAY-EDGE-TEST.md).</t>
         </is>
@@ -646,7 +694,17 @@
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="4" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="4">
+        <f>ROUNDUP(C4/K4,0)*J4</f>
+        <v/>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Choose the Diameter 35.5mm option on the listing (Scott, 2026-10-17); clears the ~32.5 mm lit area. No Amazon source found yet.</t>
         </is>
@@ -694,7 +752,17 @@
           <t>https://www.aliexpress.us/item/3256812879331298.html</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="4" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="L5" s="4">
+        <f>ROUNDUP(C5/K5,0)*J5</f>
+        <v/>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Not a schematic part: modeled inside the display footprint. 8.5 mm is the lift the 3D assumes; the marketplace sockets' body height is NOT verified. On AliExpress choose the 7P option.</t>
         </is>
@@ -742,9 +810,18 @@
           <t>https://www.aliexpress.us/item/3256812879331298.html</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Same part as the display sockets; 7 per board in all.</t>
+      <c r="J6" s="4" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Same part as the display sockets; 7 per board in all. Build cost 0: they come out of the line above's 60-pack.</t>
         </is>
       </c>
     </row>
@@ -790,105 +867,135 @@
           <t>https://www.aliexpress.us/item/3256806779943089.html</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="4" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L7" s="4">
+        <f>ROUNDUP(C7/K7,0)*J7</f>
+        <v/>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Soldered to the XIAO, plugs into the XIAO sockets. Skip if the XIAO was bought Pre-Soldered.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>SW1-SW3</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Tactile switch, right angle, 6x6 mm</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>SPST-NO, through hole, side actuated</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>SW_Tactile_SPST_Angled_PTS645Vx39-2LFS</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>C&amp;K PTS645VL39-2 LFS (footprint part)</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B008DS13P2</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256810140983087.html</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="7" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="L8" s="7">
+        <f>ROUNDUP(C8/K8,0)*J8</f>
+        <v/>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>FIT NOT VERIFIED: the footprint is the C&amp;K part (7.0 mm mounting-pin pitch); the uxcell 6x6x8 on Amazon lists 6.5 mm. Check one against the board before buying a lot. Exact part: https://lcsc.com/product-detail/Tactile-Switches_C-K-PTS645VL392LFS_C285523.html</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Electrolytic capacitor, +5V bulk</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>VALUE NOT IN SCHEMATIC - suggested 100 uF 16 V, 6.3 mm dia, 2.5 mm pitch</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Electrolytic capacitor 100 uF 16 V, +5V bulk</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>100 uF 16 V, 6.3 mm dia, 2.5 mm pitch</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>CP_Radial_D6.3mm_P2.50mm</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Panasonic EEU-FC1C101H (suggested)</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Panasonic EEU-FC1C101H (reference)</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>https://www.amazon.com/dp/B0CPDF3HHB</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>https://www.aliexpress.us/item/3256812824344961.html</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>Schematic Value field holds the symbol name only - pick and record a value. The Amazon kit lists no dimensions: check 6.3 mm dia / 2.5 mm pitch. AliExpress is Nichicon 6.3x7. Height is on the back side; check enclosure clearance.</t>
+      <c r="J9" s="7" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="L9" s="7">
+        <f>ROUNDUP(C9/K9,0)*J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Value set by Scott 2026-10-17 and now in the schematic. The Amazon listing gives no size, so 6.3 mm dia / 2.5 mm pitch is NOT VERIFIED for it; AliExpress is Nichicon 6.3x7. Height is on the back side; check enclosure clearance.</t>
         </is>
       </c>
     </row>
@@ -934,7 +1041,17 @@
           <t>https://www.aliexpress.us/item/3256811560978404.html</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="4" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="L10" s="4">
+        <f>ROUNDUP(C10/K10,0)*J10</f>
+        <v/>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Display RST hold-off with R1. Both listings are 5.08 mm pitch.</t>
         </is>
@@ -982,7 +1099,17 @@
           <t>https://www.aliexpress.us/item/3256807898146236.html</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="4" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L11" s="4">
+        <f>ROUNDUP(C11/K11,0)*J11</f>
+        <v/>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Display RST pull-up to 3V3.</t>
         </is>
@@ -1030,7 +1157,17 @@
           <t>https://www.aliexpress.us/item/3256805704775238.html</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="4" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="L12" s="4">
+        <f>ROUNDUP(C12/K12,0)*J12</f>
+        <v/>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Standoffs/length set by the enclosure, not chosen yet.</t>
         </is>
@@ -1078,14 +1215,49 @@
           <t>https://www.pcbway.com/</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Order the colors explicitly: the stackup colors only drive the 3D/STEP, not the gerbers.</t>
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Total, one build</t>
+        </is>
+      </c>
+      <c r="L15" s="9">
+        <f>SUM(L2:L13)</f>
+        <v/>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Link 1 prices seen 2026-10-17, before shipping and tax. PCB not included: get a JLCPCB quote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Per-board share</t>
+        </is>
+      </c>
+      <c r="L16" s="9">
+        <f>C2/K2*J2+C3/K3*J3+C4/K4*J4+C5/K5*J5+C6/K6*J6+C7/K7*J7+C8/K8*J8+C9/K9*J9+C10/K10*J10+C11/K11*J11+C12/K12*J12</f>
+        <v/>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Each pack pro-rated over the boards it covers.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J13"/>
+  <autoFilter ref="A1:M13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>

</xml_diff>

<commit_message>
bom: C1 Amazon link states its size; styled xlsx
C1's Amazon 50-pack (B0CPDF3HHB) never stated a size, which is why the
line stayed flagged. Swapped Link 1 to iProtool 6.3x11 mm (B0992PZC82,
$6.60/10). Neither listing states pitch; 6.3 mm radials are 2.5 mm by
convention, so the flag is dropped and the note says that is the basis.
Rejected the 5x11 mm parts that dominate Amazon results: 5 mm cans are
2.0 mm pitch and the footprint is 6.3/2.5. Totals now $105.61 one build,
$56.13 per-board share.

xlsx gets a navy header, banded rows, thin rules, vendor names as link
text instead of bare URLs, and a shaded totals block. Flagged lines keep
the yellow fill AND the NOT VERIFIED words, so the flag never depends
on color alone. The csv keeps raw URLs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
+++ b/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,13 +31,21 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -46,7 +54,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="001F3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -54,8 +67,13 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -63,33 +81,83 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D7DE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,6 +520,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F3A5F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -465,15 +534,15 @@
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -544,7 +613,7 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>U2</t>
         </is>
@@ -552,105 +621,105 @@
       <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Seeed Studio XIAO ESP32-S3</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>ESP32-S3R8, 8 MB flash, 8 MB PSRAM; SKU 113991114</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>XIAO-ESP32-S3-SOCKET</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>113991114</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.seeedstudio.com/XIAO-ESP32S3-p-5627.html</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0BYSB66S5</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="n">
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Seeed</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n">
         <v>7.49</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="6">
         <f>ROUNDUP(C2/K2,0)*J2</f>
         <v/>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Primary. Seeed sells it with pin headers Un-Soldered or Pre-Soldered; Pre-Soldered makes the male header line below unnecessary. ALTERNATE if more memory is wanted: XIAO ESP32-S3 Plus (16 MB flash, SKU 102010671) https://www.seeedstudio.com/Seeed-Studio-XIAO-ESP32S3-Plus-p-6361.html / https://www.amazon.com/dp/B0H6XJGN3Z / https://www.aliexpress.us/item/3256808599305867.html - ships WITHOUT headers. Same footprint and the same 8 MB firmware binary on both. Mounted on the back, on sockets.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>DS1-DS5</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>1.28in round TFT, GC9A01, 240x240, 7-pin SPI</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>7-pin 2.54 mm header, order VCC GND SCL SDA DC CS RST</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>_Displays:GC9A01_SOCKET</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>generic</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJ13VW73</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256813175276825.html</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="n">
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="n">
         <v>17.99</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="11">
         <f>ROUNDUP(C3/K3,0)*J3</f>
         <v/>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>Check the listing's pin order before buying; the footprint is pad 1 = VCC (+5V) .. pad 7 = RST. The module's own male header plugs into the female socket below. Lit area ~32.5 mm dia (docs/DISPLAY-EDGE-TEST.md).</t>
         </is>
@@ -660,7 +729,7 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>LENS1-LENS5</t>
         </is>
@@ -668,101 +737,101 @@
       <c r="C4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Display lens: mineral watch crystal, double dome</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>35.5 mm dia, 2.0 mm thick</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>enclosure part, no footprint</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>generic</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256806569387664.html</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="4" t="n">
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="6" t="n">
         <v>3.08</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="6">
         <f>ROUNDUP(C4/K4,0)*J4</f>
         <v/>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Choose the Diameter 35.5mm option on the listing (Scott, 2026-10-17); clears the ~32.5 mm lit area. No Amazon source found yet.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>J (displays)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Female socket 1x07, 2.54 mm, straight</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>8.5 mm body, through hole</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>PinSocket_1x07_P2.54mm_Vertical (in GC9A01_SOCKET)</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Sullins PPTC071LFBN-RC (reference)</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0GM7T6XWP</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256812879331298.html</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="n">
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="n">
         <v>6.99</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="11">
         <f>ROUNDUP(C5/K5,0)*J5</f>
         <v/>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>Not a schematic part: modeled inside the display footprint. 8.5 mm is the lift the 3D assumes; the marketplace sockets' body height is NOT verified. On AliExpress choose the 7P option.</t>
         </is>
@@ -772,7 +841,7 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>J (XIAO)</t>
         </is>
@@ -780,222 +849,222 @@
       <c r="C6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Female socket 1x07, 2.54 mm, straight</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>8.5 mm body, through hole</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>in XIAO-ESP32-S3-SOCKET</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Sullins PPTC071LFBN-RC (reference)</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0GM7T6XWP</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256812879331298.html</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="n">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n">
         <v>6.99</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="L6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Same part as the display sockets; 7 per board in all. Build cost 0: they come out of the line above's 60-pack.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>P (XIAO)</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Male header 1x07, 2.54 mm</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>cut from a 1x40 breakaway strip (1 strip = 5 sets)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>in XIAO-ESP32-S3-SOCKET</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Sullins PRPC040SAAN-RC (reference)</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0FRZW75VS</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256806779943089.html</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="n">
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="n">
         <v>6.29</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="L7" s="4">
+      <c r="L7" s="11">
         <f>ROUNDUP(C7/K7,0)*J7</f>
         <v/>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>Soldered to the XIAO, plugs into the XIAO sockets. Skip if the XIAO was bought Pre-Soldered.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>SW1-SW3</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Tactile switch, right angle, 6x6 mm</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>SPST-NO, through hole, side actuated</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>SW_Tactile_SPST_Angled_PTS645Vx39-2LFS</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>C&amp;K PTS645VL39-2 LFS (footprint part)</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B008DS13P2</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256810140983087.html</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="n">
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="n">
         <v>7.39</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="16">
         <f>ROUNDUP(C8/K8,0)*J8</f>
         <v/>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="M8" s="14" t="inlineStr">
         <is>
           <t>FIT NOT VERIFIED: the footprint is the C&amp;K part (7.0 mm mounting-pin pitch); the uxcell 6x6x8 on Amazon lists 6.5 mm. Check one against the board before buying a lot. Exact part: https://lcsc.com/product-detail/Tactile-Switches_C-K-PTS645VL392LFS_C285523.html</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Electrolytic capacitor 100 uF 16 V, +5V bulk</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>100 uF 16 V, 6.3 mm dia, 2.5 mm pitch</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>CP_Radial_D6.3mm_P2.50mm</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Panasonic EEU-FC1C101H (reference)</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CPDF3HHB</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256812824344961.html</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="K9" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="L9" s="7">
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="L9" s="11">
         <f>ROUNDUP(C9/K9,0)*J9</f>
         <v/>
       </c>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>Value set by Scott 2026-10-17 and now in the schematic. The Amazon listing gives no size, so 6.3 mm dia / 2.5 mm pitch is NOT VERIFIED for it; AliExpress is Nichicon 6.3x7. Height is on the back side; check enclosure clearance.</t>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Value set by Scott 2026-10-17. Both listings state 6.3 mm dia (Amazon 6.3x11, AliExpress Nichicon 6.3x7); neither states pitch, and 6.3 mm radials are 2.5 mm by convention. Mounted on the back: the 11 mm Amazon part stands 4 mm taller than the AliExpress one, so check enclosure clearance.</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1072,7 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
@@ -1011,105 +1080,105 @@
       <c r="C10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Ceramic capacitor 1 uF (105)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>50 V, radial, 5.08 mm lead spacing</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>C_Disc_D5.0mm_W2.5mm_P5.00mm</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>KEMET C330C105K5R5TA7301 (reference)</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B08BF91KY3</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256811560978404.html</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="n">
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n">
         <v>6.99</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="6">
         <f>ROUNDUP(C10/K10,0)*J10</f>
         <v/>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>Display RST hold-off with R1. Both listings are 5.08 mm pitch.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Resistor 10k</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>1/4 W 5 % carbon film, axial, 10.16 mm pitch</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>Stackpole CF14JT10K0 (reference)</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0CL9KXXZB</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256807898146236.html</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="n">
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="n">
         <v>4.99</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11" s="11">
         <f>ROUNDUP(C11/K11,0)*J11</f>
         <v/>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M11" s="9" t="inlineStr">
         <is>
           <t>Display RST pull-up to 3V3.</t>
         </is>
@@ -1119,7 +1188,7 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>H1-H7</t>
         </is>
@@ -1127,130 +1196,130 @@
       <c r="C12" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>M3 screw (mounting)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>M3-0.5, socket head; 3.2 mm holes</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Edge.Cuts circles, no footprint</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>M3 x 6 DIN 912 class 12.9 (length depends on the enclosure)</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amazon.com/dp/B0DJQH3WSX</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256805704775238.html</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="n">
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="n">
         <v>7.49</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12" s="6">
         <f>ROUNDUP(C12/K12,0)*J12</f>
         <v/>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>Standoffs/length set by the enclosure, not chosen yet.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C13" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Bare board</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>2 layer, 1.6 mm, 198.82 x 47.78 mm, WHITE solder mask, BLACK silkscreen</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>hot_info_orbs_xiao.kicad_pcb</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>https://jlcpcb.com/quote/pcbOrderFaq/PCB%20Color</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.pcbway.com/</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>PCBWay</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="11" t="inlineStr"/>
+      <c r="M13" s="9" t="inlineStr">
         <is>
           <t>Order the colors explicitly: the stackup colors only drive the 3D/STEP, not the gerbers.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="K15" s="8" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>Total, one build</t>
         </is>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="18">
         <f>SUM(L2:L13)</f>
         <v/>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M15" s="19" t="inlineStr">
         <is>
           <t>Link 1 prices seen 2026-10-17, before shipping and tax. PCB not included: get a JLCPCB quote.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="K16" s="8" t="inlineStr">
+      <c r="K16" s="17" t="inlineStr">
         <is>
           <t>Per-board share</t>
         </is>
       </c>
-      <c r="L16" s="9">
+      <c r="L16" s="18">
         <f>C2/K2*J2+C3/K3*J3+C4/K4*J4+C5/K5*J5+C6/K6*J6+C7/K7*J7+C8/K8*J8+C9/K9*J9+C10/K10*J10+C11/K11*J11+C12/K12*J12</f>
         <v/>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M16" s="19" t="inlineStr">
         <is>
           <t>Each pack pro-rated over the boards it covers.</t>
         </is>

</xml_diff>

<commit_message>
bom: lenses optional (glass + laser-cut acrylic, TBD); options under totals
Scott 2026-10-17: lenses are likely optional, and an acrylic disc cut on
the laser may be offered. Glass and acrylic are now two OPTIONAL lines
kept off the build totals and priced as option rows under them: glass
$15.40 per board, acrylic TBD. Required build: $90.21 whole packs,
$40.73 per-board share.

Also answers "did you count both ESPs": only one XIAO was ever costed
(plain S3, $7.49). The Plus ($7.90 on Seeed, seen today) replaces it, so
it gets an option row (+$0.41) rather than a BOM line, which would have
double-counted the module.

Option labels say "Option:" instead of a leading "+": Sheets parsed
"+ Glass..." as a formula and showed #ERROR!.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
+++ b/hardware/hot-info-orbs-xiao/bom/hot_info_orbs_xiao_bom.xlsx
@@ -10,7 +10,7 @@
     <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$M$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,12 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -99,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,7 +123,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -132,7 +138,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -147,7 +153,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -156,6 +162,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -524,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -731,7 +743,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>LENS1-LENS5</t>
+          <t>LENS1-LENS5 (glass)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -775,7 +787,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>Choose the Diameter 35.5mm option on the listing (Scott, 2026-10-17); clears the ~32.5 mm lit area. No Amazon source found yet.</t>
+          <t>OPTIONAL, not in the build total (priced as an add-on below it). Choose the Diameter 35.5mm option on the listing (Scott, 2026-10-17); clears the ~32.5 mm lit area. No Amazon source found yet.</t>
         </is>
       </c>
     </row>
@@ -785,7 +797,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>J (displays)</t>
+          <t>LENS1-LENS5 (acrylic)</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
@@ -793,47 +805,46 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Female socket 1x07, 2.54 mm, straight</t>
+          <t>Display lens: laser-cut clear acrylic disc</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>8.5 mm body, through hole</t>
+          <t>35.5 mm dia, thickness TBD</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>PinSocket_1x07_P2.54mm_Vertical (in GC9A01_SOCKET)</t>
+          <t>enclosure part, no footprint</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Sullins PPTC071LFBN-RC (reference)</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>6.99</v>
+          <t>cut in-house</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>in-house (laser)</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr"/>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
       </c>
       <c r="K5" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="L5" s="11">
-        <f>ROUNDUP(C5/K5,0)*J5</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>Not a schematic part: modeled inside the display footprint. 8.5 mm is the lift the 3D assumes; the marketplace sockets' body height is NOT verified. On AliExpress choose the 7P option.</t>
+          <t>OPTIONAL alternative to the glass lens, price TBD (Scott, 2026-10-17). Flat, so no dome. Same 35.5 mm diameter as the glass; the bezel has to allow for whichever thickness is chosen.</t>
         </is>
       </c>
     </row>
@@ -843,11 +854,11 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>J (XIAO)</t>
+          <t>J (displays)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -861,7 +872,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>in XIAO-ESP32-S3-SOCKET</t>
+          <t>PinSocket_1x07_P2.54mm_Vertical (in GC9A01_SOCKET)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -885,12 +896,13 @@
       <c r="K6" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="L6" s="6" t="n">
-        <v>0</v>
+      <c r="L6" s="6">
+        <f>ROUNDUP(C6/K6,0)*J6</f>
+        <v/>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>Same part as the display sockets; 7 per board in all. Build cost 0: they come out of the line above's 60-pack.</t>
+          <t>Not a schematic part: modeled inside the display footprint. 8.5 mm is the lift the 3D assumes; the marketplace sockets' body height is NOT verified. On AliExpress choose the 7P option.</t>
         </is>
       </c>
     </row>
@@ -900,7 +912,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>P (XIAO)</t>
+          <t>J (XIAO)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
@@ -908,163 +920,162 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
+          <t>Female socket 1x07, 2.54 mm, straight</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>8.5 mm body, through hole</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>in XIAO-ESP32-S3-SOCKET</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Sullins PPTC071LFBN-RC (reference)</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>Same part as the display sockets; 7 per board in all. Build cost 0: they come out of the line above's 60-pack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>P (XIAO)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
           <t>Male header 1x07, 2.54 mm</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>cut from a 1x40 breakaway strip (1 strip = 5 sets)</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>in XIAO-ESP32-S3-SOCKET</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Sullins PRPC040SAAN-RC (reference)</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="J7" s="11" t="n">
+      <c r="J8" s="6" t="n">
         <v>6.29</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="K8" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="L7" s="11">
-        <f>ROUNDUP(C7/K7,0)*J7</f>
-        <v/>
-      </c>
-      <c r="M7" s="9" t="inlineStr">
-        <is>
-          <t>Soldered to the XIAO, plugs into the XIAO sockets. Skip if the XIAO was bought Pre-Soldered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>SW1-SW3</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Tactile switch, right angle, 6x6 mm</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>SPST-NO, through hole, side actuated</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>SW_Tactile_SPST_Angled_PTS645Vx39-2LFS</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="inlineStr">
-        <is>
-          <t>C&amp;K PTS645VL39-2 LFS (footprint part)</t>
-        </is>
-      </c>
-      <c r="H8" s="15" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
-      <c r="J8" s="16" t="n">
-        <v>7.39</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="L8" s="16">
+      <c r="L8" s="6">
         <f>ROUNDUP(C8/K8,0)*J8</f>
         <v/>
       </c>
-      <c r="M8" s="14" t="inlineStr">
-        <is>
-          <t>FIT NOT VERIFIED: the footprint is the C&amp;K part (7.0 mm mounting-pin pitch); the uxcell 6x6x8 on Amazon lists 6.5 mm. Check one against the board before buying a lot. Exact part: https://lcsc.com/product-detail/Tactile-Switches_C-K-PTS645VL392LFS_C285523.html</t>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>Soldered to the XIAO, plugs into the XIAO sockets. Skip if the XIAO was bought Pre-Soldered.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Electrolytic capacitor 100 uF 16 V, +5V bulk</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>100 uF 16 V, 6.3 mm dia, 2.5 mm pitch</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>CP_Radial_D6.3mm_P2.50mm</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Panasonic EEU-FC1C101H (reference)</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>SW1-SW3</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Tactile switch, right angle, 6x6 mm</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>SPST-NO, through hole, side actuated</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>SW_Tactile_SPST_Angled_PTS645Vx39-2LFS</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>C&amp;K PTS645VL39-2 LFS (footprint part)</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="15" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="J9" s="11" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="L9" s="11">
+      <c r="J9" s="16" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="L9" s="16">
         <f>ROUNDUP(C9/K9,0)*J9</f>
         <v/>
       </c>
-      <c r="M9" s="9" t="inlineStr">
-        <is>
-          <t>Value set by Scott 2026-10-17. Both listings state 6.3 mm dia (Amazon 6.3x11, AliExpress Nichicon 6.3x7); neither states pitch, and 6.3 mm radials are 2.5 mm by convention. Mounted on the back: the 11 mm Amazon part stands 4 mm taller than the AliExpress one, so check enclosure clearance.</t>
+      <c r="M9" s="14" t="inlineStr">
+        <is>
+          <t>FIT NOT VERIFIED: the footprint is the C&amp;K part (7.0 mm mounting-pin pitch); the uxcell 6x6x8 on Amazon lists 6.5 mm. Check one against the board before buying a lot. Exact part: https://lcsc.com/product-detail/Tactile-Switches_C-K-PTS645VL392LFS_C285523.html</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1085,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1082,22 +1093,22 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Ceramic capacitor 1 uF (105)</t>
+          <t>Electrolytic capacitor 100 uF 16 V, +5V bulk</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>50 V, radial, 5.08 mm lead spacing</t>
+          <t>100 uF 16 V, 6.3 mm dia, 2.5 mm pitch</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>C_Disc_D5.0mm_W2.5mm_P5.00mm</t>
+          <t>CP_Radial_D6.3mm_P2.50mm</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>KEMET C330C105K5R5TA7301 (reference)</t>
+          <t>Panasonic EEU-FC1C101H (reference)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1111,10 +1122,10 @@
         </is>
       </c>
       <c r="J10" s="6" t="n">
-        <v>6.99</v>
+        <v>6.6</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="L10" s="6">
         <f>ROUNDUP(C10/K10,0)*J10</f>
@@ -1122,7 +1133,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>Display RST hold-off with R1. Both listings are 5.08 mm pitch.</t>
+          <t>Value set by Scott 2026-10-17. Both listings state 6.3 mm dia (Amazon 6.3x11, AliExpress Nichicon 6.3x7); neither states pitch, and 6.3 mm radials are 2.5 mm by convention. Mounted on the back: the 11 mm Amazon part stands 4 mm taller than the AliExpress one, so check enclosure clearance.</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1143,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
@@ -1140,22 +1151,22 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Resistor 10k</t>
+          <t>Ceramic capacitor 1 uF (105)</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>1/4 W 5 % carbon film, axial, 10.16 mm pitch</t>
+          <t>50 V, radial, 5.08 mm lead spacing</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
+          <t>C_Disc_D5.0mm_W2.5mm_P5.00mm</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Stackpole CF14JT10K0 (reference)</t>
+          <t>KEMET C330C105K5R5TA7301 (reference)</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
@@ -1169,10 +1180,10 @@
         </is>
       </c>
       <c r="J11" s="11" t="n">
-        <v>4.99</v>
+        <v>6.99</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="L11" s="11">
         <f>ROUNDUP(C11/K11,0)*J11</f>
@@ -1180,7 +1191,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>Display RST pull-up to 3V3.</t>
+          <t>Display RST hold-off with R1. Both listings are 5.08 mm pitch.</t>
         </is>
       </c>
     </row>
@@ -1190,30 +1201,30 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>H1-H7</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>M3 screw (mounting)</t>
+          <t>Resistor 10k</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>M3-0.5, socket head; 3.2 mm holes</t>
+          <t>1/4 W 5 % carbon film, axial, 10.16 mm pitch</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Edge.Cuts circles, no footprint</t>
+          <t>R_Axial_DIN0207_L6.3mm_D2.5mm_P10.16mm_Horizontal</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>M3 x 6 DIN 912 class 12.9 (length depends on the enclosure)</t>
+          <t>Stackpole CF14JT10K0 (reference)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1227,10 +1238,10 @@
         </is>
       </c>
       <c r="J12" s="6" t="n">
-        <v>7.49</v>
+        <v>4.99</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="L12" s="6">
         <f>ROUNDUP(C12/K12,0)*J12</f>
@@ -1238,7 +1249,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>Standoffs/length set by the enclosure, not chosen yet.</t>
+          <t>Display RST pull-up to 3V3.</t>
         </is>
       </c>
     </row>
@@ -1248,109 +1259,216 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
+          <t>H1-H7</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>M3 screw (mounting)</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>M3-0.5, socket head; 3.2 mm holes</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Edge.Cuts circles, no footprint</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>M3 x 6 DIN 912 class 12.9 (length depends on the enclosure)</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="L13" s="11">
+        <f>ROUNDUP(C13/K13,0)*J13</f>
+        <v/>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>Standoffs/length set by the enclosure, not chosen yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Bare board</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>2 layer, 1.6 mm, 198.82 x 47.78 mm, WHITE solder mask, BLACK silkscreen</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>hot_info_orbs_xiao.kicad_pcb</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>PCBWay</t>
         </is>
       </c>
-      <c r="J13" s="11" t="inlineStr"/>
-      <c r="K13" s="7" t="inlineStr"/>
-      <c r="L13" s="11" t="inlineStr"/>
-      <c r="M13" s="9" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Order the colors explicitly: the stackup colors only drive the 3D/STEP, not the gerbers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="K15" s="17" t="inlineStr">
-        <is>
-          <t>Total, one build</t>
-        </is>
-      </c>
-      <c r="L15" s="18">
-        <f>SUM(L2:L13)</f>
-        <v/>
-      </c>
-      <c r="M15" s="19" t="inlineStr">
-        <is>
-          <t>Link 1 prices seen 2026-10-17, before shipping and tax. PCB not included: get a JLCPCB quote.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="K16" s="17" t="inlineStr">
         <is>
+          <t>Total, one build</t>
+        </is>
+      </c>
+      <c r="L16" s="18">
+        <f>L2+L3+L6+L7+L8+L9+L10+L11+L12+L13</f>
+        <v/>
+      </c>
+      <c r="M16" s="19" t="inlineStr">
+        <is>
+          <t>Required lines only; the optional lenses are below. Link 1 prices seen 2026-10-17, before shipping and tax. PCB not included: get a JLCPCB quote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="K17" s="17" t="inlineStr">
+        <is>
           <t>Per-board share</t>
         </is>
       </c>
-      <c r="L16" s="18">
-        <f>C2/K2*J2+C3/K3*J3+C4/K4*J4+C5/K5*J5+C6/K6*J6+C7/K7*J7+C8/K8*J8+C9/K9*J9+C10/K10*J10+C11/K11*J11+C12/K12*J12</f>
+      <c r="L17" s="18">
+        <f>C2/K2*J2+C3/K3*J3+C6/K6*J6+C7/K7*J7+C8/K8*J8+C9/K9*J9+C10/K10*J10+C11/K11*J11+C12/K12*J12+C13/K13*J13</f>
         <v/>
       </c>
-      <c r="M16" s="19" t="inlineStr">
+      <c r="M17" s="19" t="inlineStr">
         <is>
           <t>Each pack pro-rated over the boards it covers.</t>
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>Option: glass lenses, per board</t>
+        </is>
+      </c>
+      <c r="L18" s="21">
+        <f>L4</f>
+        <v/>
+      </c>
+      <c r="M18" s="19" t="inlineStr">
+        <is>
+          <t>Five watch crystals, one per display.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>Option: acrylic lenses, per board</t>
+        </is>
+      </c>
+      <c r="L19" s="21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="M19" s="19" t="inlineStr">
+        <is>
+          <t>Laser-cut in-house; price not set yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>Option: S3 Plus instead of S3, per board</t>
+        </is>
+      </c>
+      <c r="L20" s="21">
+        <f>7.9-J2</f>
+        <v/>
+      </c>
+      <c r="M20" s="19" t="inlineStr">
+        <is>
+          <t>The Plus ($7.90 on Seeed, seen 2026-10-17) REPLACES U2; only one XIAO goes on a board.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M13"/>
+  <autoFilter ref="A1:M14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>